<commit_message>
fix: rename deliverables to AuthorYear_Report.xlsx, add PDF generation for all 10 papers
- Updated author_year for papers 0018-0025: AntiCorruption->Fang2022,
  AntidiscrimLaws->Greene2021, CompetingAttention->Meyer2024,
  CorporateBoards->Hu2025, DemandPull->Santamaria2024, EffectIPO->Chyz2023,
  HedingHill->Christensen2021, PathwaysProfits->Anderson2018
- Renamed output from AuthorYearReport_{id}.xlsx to {AuthorYear}_Report.xlsx
- Added generate_paper_info_pdf() using reportlab — generates Paper_Info_Record.pdf
  matching RA_MISSING_DATA.pdf Appendix A (6 sections) for all 10 papers
- Updated paper_info xlsx files with real author names and journal/year info
- Generated all 10 {AuthorYear}_Report.xlsx workbooks and Paper_Info_Record PDFs

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/paper_analysis_output/Paper_0005_MappingEntrepreneurial/smoke/SMOKE_Stroube2025Report_0005.xlsx
+++ b/paper_analysis_output/Paper_0005_MappingEntrepreneurial/smoke/SMOKE_Stroube2025Report_0005.xlsx
@@ -713,10 +713,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D2" t="n">
         <v>100</v>
@@ -3037,16 +3037,16 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>2.266686829980565</v>
+        <v>2.355200235794877</v>
       </c>
       <c r="G4" t="n">
-        <v>1.780918207901517</v>
+        <v>1.912724958715843</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9877300613496932</v>
+        <v>0.9938650306748467</v>
       </c>
       <c r="I4" t="n">
-        <v>0.002517123858364543</v>
+        <v>0.03068731061408272</v>
       </c>
     </row>
     <row r="5">
@@ -3111,16 +3111,16 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>2.126366132869848</v>
+        <v>2.250340105265568</v>
       </c>
       <c r="G6" t="n">
-        <v>1.678528622957997</v>
+        <v>1.711460626029377</v>
       </c>
       <c r="H6" t="n">
-        <v>0.9938650306748467</v>
+        <v>0.9846625766871165</v>
       </c>
       <c r="I6" t="n">
-        <v>0.01155631830681614</v>
+        <v>0.01997417035152385</v>
       </c>
     </row>
     <row r="7">
@@ -3148,16 +3148,16 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>3.079774391081314</v>
+        <v>2.095574915908864</v>
       </c>
       <c r="G7" t="n">
-        <v>2.655410077347826</v>
+        <v>1.701714302164703</v>
       </c>
       <c r="H7" t="n">
-        <v>0.9938650306748467</v>
+        <v>0.9969325153374233</v>
       </c>
       <c r="I7" t="n">
-        <v>7.830109917507268e-05</v>
+        <v>0.04211618495493517</v>
       </c>
     </row>
     <row r="8">
@@ -3399,16 +3399,16 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>3.215751687406613</v>
+        <v>2.160430402647616</v>
       </c>
       <c r="G14" t="n">
-        <v>2.774986735074858</v>
+        <v>1.765709255891299</v>
       </c>
       <c r="H14" t="n">
-        <v>0.9938650306748467</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>0.0004097822052991821</v>
+        <v>0.01105520232529481</v>
       </c>
     </row>
     <row r="15">
@@ -3650,16 +3650,16 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>3.08150079571877</v>
+        <v>2.286455361685413</v>
       </c>
       <c r="G21" t="n">
-        <v>2.676441786587687</v>
+        <v>1.821594432834647</v>
       </c>
       <c r="H21" t="n">
-        <v>0.9932598039215687</v>
+        <v>0.9935661764705882</v>
       </c>
       <c r="I21" t="n">
-        <v>9.105212606274726e-05</v>
+        <v>0.07979417039776898</v>
       </c>
     </row>
     <row r="22">
@@ -3901,16 +3901,16 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>3.10552239234311</v>
+        <v>2.202525422401299</v>
       </c>
       <c r="G28" t="n">
-        <v>2.705988936812309</v>
+        <v>1.732570748831836</v>
       </c>
       <c r="H28" t="n">
-        <v>0.9911151960784313</v>
+        <v>0.9905024509803921</v>
       </c>
       <c r="I28" t="n">
-        <v>2.985952750305446e-05</v>
+        <v>0.03458337575137135</v>
       </c>
     </row>
     <row r="29">
@@ -4152,16 +4152,16 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>3.059370347715736</v>
+        <v>2.222314638171643</v>
       </c>
       <c r="G35" t="n">
-        <v>2.61285933106767</v>
+        <v>1.729569478590514</v>
       </c>
       <c r="H35" t="n">
-        <v>0.9846625766871165</v>
+        <v>1</v>
       </c>
       <c r="I35" t="n">
-        <v>0.002665303919505906</v>
+        <v>0.2940216577369589</v>
       </c>
     </row>
     <row r="36">
@@ -4403,16 +4403,16 @@
         <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>3.134420276728176</v>
+        <v>2.069701633475419</v>
       </c>
       <c r="G42" t="n">
-        <v>2.682767341807123</v>
+        <v>1.666301719422746</v>
       </c>
       <c r="H42" t="n">
-        <v>0.9877300613496932</v>
+        <v>1</v>
       </c>
       <c r="I42" t="n">
-        <v>0.001192332114735274</v>
+        <v>0.07519147922064397</v>
       </c>
     </row>
     <row r="43">
@@ -4654,16 +4654,16 @@
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>3.160524989685337</v>
+        <v>2.196290654007407</v>
       </c>
       <c r="G49" t="n">
-        <v>2.752866705666809</v>
+        <v>1.745381564025054</v>
       </c>
       <c r="H49" t="n">
-        <v>0.9911151960784313</v>
+        <v>0.9950980392156863</v>
       </c>
       <c r="I49" t="n">
-        <v>0.01989854652749444</v>
+        <v>0.1438117796236238</v>
       </c>
     </row>
     <row r="50">
@@ -4905,16 +4905,16 @@
         <v>1</v>
       </c>
       <c r="F56" t="n">
-        <v>3.156494033175002</v>
+        <v>2.188469464998288</v>
       </c>
       <c r="G56" t="n">
-        <v>2.738542193495721</v>
+        <v>1.748123605352092</v>
       </c>
       <c r="H56" t="n">
-        <v>0.9898897058823529</v>
+        <v>0.9947916666666666</v>
       </c>
       <c r="I56" t="n">
-        <v>0.016937426344706</v>
+        <v>0.1295430711686345</v>
       </c>
     </row>
     <row r="57">
@@ -5156,16 +5156,16 @@
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>4.099298699313662</v>
+        <v>1.969422687008938</v>
       </c>
       <c r="G63" t="n">
-        <v>3.746991670487342</v>
+        <v>1.590369548078191</v>
       </c>
       <c r="H63" t="n">
-        <v>0.9263803680981595</v>
+        <v>1</v>
       </c>
       <c r="I63" t="n">
-        <v>0.01105299277510696</v>
+        <v>0.8696421309245648</v>
       </c>
     </row>
     <row r="64">
@@ -5407,16 +5407,16 @@
         <v>1</v>
       </c>
       <c r="F70" t="n">
-        <v>4.020010851939074</v>
+        <v>2.183841639073207</v>
       </c>
       <c r="G70" t="n">
-        <v>3.65694518615938</v>
+        <v>1.820310888981146</v>
       </c>
       <c r="H70" t="n">
-        <v>0.9386503067484663</v>
+        <v>1</v>
       </c>
       <c r="I70" t="n">
-        <v>0.01055079016517099</v>
+        <v>0.7307167558707346</v>
       </c>
     </row>
     <row r="71">
@@ -5658,16 +5658,16 @@
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>4.225725889395394</v>
+        <v>2.377212995031329</v>
       </c>
       <c r="G77" t="n">
-        <v>3.877498966580898</v>
+        <v>1.930755247705656</v>
       </c>
       <c r="H77" t="n">
-        <v>0.9255514705882353</v>
+        <v>0.9923406862745098</v>
       </c>
       <c r="I77" t="n">
-        <v>0.1182437936832994</v>
+        <v>0.6444939383049477</v>
       </c>
     </row>
     <row r="78">
@@ -5909,16 +5909,16 @@
         <v>1</v>
       </c>
       <c r="F84" t="n">
-        <v>4.271998755607784</v>
+        <v>2.226816640650056</v>
       </c>
       <c r="G84" t="n">
-        <v>3.926878178629635</v>
+        <v>1.788477134372259</v>
       </c>
       <c r="H84" t="n">
-        <v>0.9175857843137255</v>
+        <v>0.9935661764705882</v>
       </c>
       <c r="I84" t="n">
-        <v>0.120358453130825</v>
+        <v>0.7345148268818036</v>
       </c>
     </row>
     <row r="85">
@@ -6118,16 +6118,16 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0013</v>
+        <v>0.0015</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0003</v>
+        <v>-0.0007</v>
       </c>
       <c r="I4" t="n">
-        <v>1.0005</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="5">
@@ -6198,7 +6198,7 @@
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.0001</v>
+        <v>-0.0004</v>
       </c>
       <c r="I6" t="n">
         <v>1.0002</v>
@@ -6229,16 +6229,16 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0051</v>
+        <v>0.0014</v>
       </c>
       <c r="G7" t="n">
-        <v>0.7905</v>
+        <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0002</v>
+        <v>-0.0011</v>
       </c>
       <c r="I7" t="n">
-        <v>0.995</v>
+        <v>0.9998</v>
       </c>
     </row>
     <row r="8">
@@ -6488,16 +6488,16 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0053</v>
+        <v>0.0015</v>
       </c>
       <c r="G14" t="n">
-        <v>0.7533</v>
+        <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.0013</v>
+        <v>-0.0009</v>
       </c>
       <c r="I14" t="n">
-        <v>0.9946</v>
+        <v>0.9991</v>
       </c>
     </row>
     <row r="15">
@@ -6747,16 +6747,16 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>0.0503</v>
+        <v>0.0139</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>0.0036</v>
       </c>
       <c r="H21" t="n">
-        <v>0.0003</v>
+        <v>-0.0245</v>
       </c>
       <c r="I21" t="n">
-        <v>0.9492</v>
+        <v>0.9965000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -7006,16 +7006,16 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>0.0507</v>
+        <v>0.0138</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="H28" t="n">
-        <v>0.0001</v>
+        <v>-0.0106</v>
       </c>
       <c r="I28" t="n">
-        <v>0.9484</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="29">
@@ -7265,16 +7265,16 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>0.0064</v>
+        <v>0.001</v>
       </c>
       <c r="G35" t="n">
-        <v>0.5194</v>
+        <v>1</v>
       </c>
       <c r="H35" t="n">
-        <v>-0.0083</v>
+        <v>0.0009</v>
       </c>
       <c r="I35" t="n">
-        <v>0.9951</v>
+        <v>1.0004</v>
       </c>
     </row>
     <row r="36">
@@ -7524,16 +7524,16 @@
         <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>0.0054</v>
+        <v>0.0013</v>
       </c>
       <c r="G42" t="n">
-        <v>0.7341</v>
+        <v>1</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.0037</v>
+        <v>-0.0013</v>
       </c>
       <c r="I42" t="n">
-        <v>0.9949</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="43">
@@ -7783,16 +7783,16 @@
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>0.0586</v>
+        <v>0.0113</v>
       </c>
       <c r="G49" t="n">
-        <v>0</v>
+        <v>0.03</v>
       </c>
       <c r="H49" t="n">
-        <v>-0.0616</v>
+        <v>-0.0109</v>
       </c>
       <c r="I49" t="n">
-        <v>0.9467</v>
+        <v>1.0018</v>
       </c>
     </row>
     <row r="50">
@@ -8042,16 +8042,16 @@
         <v>1</v>
       </c>
       <c r="F56" t="n">
-        <v>0.0566</v>
+        <v>0.0125</v>
       </c>
       <c r="G56" t="n">
-        <v>0</v>
+        <v>0.0118</v>
       </c>
       <c r="H56" t="n">
-        <v>-0.0525</v>
+        <v>-0.0071</v>
       </c>
       <c r="I56" t="n">
-        <v>0.9468</v>
+        <v>0.9971</v>
       </c>
     </row>
     <row r="57">
@@ -8301,16 +8301,16 @@
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>0.0092</v>
+        <v>0.0017</v>
       </c>
       <c r="G63" t="n">
-        <v>0.1262</v>
+        <v>1</v>
       </c>
       <c r="H63" t="n">
-        <v>-0.0342</v>
+        <v>-0.007</v>
       </c>
       <c r="I63" t="n">
-        <v>0.9913</v>
+        <v>0.9989</v>
       </c>
     </row>
     <row r="64">
@@ -8560,16 +8560,16 @@
         <v>1</v>
       </c>
       <c r="F70" t="n">
-        <v>0.0091</v>
+        <v>0.0022</v>
       </c>
       <c r="G70" t="n">
-        <v>0.1357</v>
+        <v>1</v>
       </c>
       <c r="H70" t="n">
-        <v>-0.0327</v>
+        <v>-0.0098</v>
       </c>
       <c r="I70" t="n">
-        <v>0.9916</v>
+        <v>0.9976</v>
       </c>
     </row>
     <row r="71">
@@ -8819,16 +8819,16 @@
         <v>0</v>
       </c>
       <c r="F77" t="n">
-        <v>0.09320000000000001</v>
+        <v>0.0271</v>
       </c>
       <c r="G77" t="n">
         <v>0</v>
       </c>
       <c r="H77" t="n">
-        <v>-0.3662</v>
+        <v>-0.13</v>
       </c>
       <c r="I77" t="n">
-        <v>0.9098000000000001</v>
+        <v>0.9727</v>
       </c>
     </row>
     <row r="78">
@@ -9078,16 +9078,16 @@
         <v>1</v>
       </c>
       <c r="F84" t="n">
-        <v>0.094</v>
+        <v>0.0228</v>
       </c>
       <c r="G84" t="n">
         <v>0</v>
       </c>
       <c r="H84" t="n">
-        <v>-0.3727</v>
+        <v>-0.108</v>
       </c>
       <c r="I84" t="n">
-        <v>0.9079</v>
+        <v>0.9767</v>
       </c>
     </row>
     <row r="85">
@@ -11770,16 +11770,16 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>34.2</v>
       </c>
       <c r="M7" t="n">
-        <v>65.8</v>
+        <v>100</v>
       </c>
       <c r="N7" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
@@ -11917,10 +11917,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.01404897885601543</v>
+        <v>0.001498574486025016</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5997981537527336</v>
+        <v>0.8394549660612634</v>
       </c>
       <c r="F2" t="n">
         <v>2</v>
@@ -11943,10 +11943,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.001706291176941912</v>
+        <v>0.0005373236586433972</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9292984011763041</v>
+        <v>1.003205523893243</v>
       </c>
       <c r="F3" t="n">
         <v>2</v>
@@ -11969,10 +11969,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.009538970885003096</v>
+        <v>0.003455509785009332</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6331205695251606</v>
+        <v>0.7817419343101325</v>
       </c>
       <c r="F4" t="n">
         <v>2</v>
@@ -11995,10 +11995,10 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.0008398464016898609</v>
+        <v>0.0001236373839479118</v>
       </c>
       <c r="E5" t="n">
-        <v>0.948419211472932</v>
+        <v>0.9862515585405308</v>
       </c>
       <c r="F5" t="n">
         <v>2</v>
@@ -12021,10 +12021,10 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.02586179918087284</v>
+        <v>0.003173952127051057</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4824174113398739</v>
+        <v>0.7409657366125879</v>
       </c>
       <c r="F6" t="n">
         <v>2</v>
@@ -12047,10 +12047,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.004597236081295625</v>
+        <v>0.0007625753075897881</v>
       </c>
       <c r="E7" t="n">
-        <v>0.819820362249672</v>
+        <v>0.9674338213942429</v>
       </c>
       <c r="F7" t="n">
         <v>2</v>
@@ -12775,10 +12775,10 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.0004104488456682813</v>
+        <v>0.0006682602276470666</v>
       </c>
       <c r="E35" t="n">
-        <v>0.9984535864722386</v>
+        <v>1.004092149888086</v>
       </c>
       <c r="F35" t="n">
         <v>2</v>
@@ -12931,10 +12931,10 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.0005449428645692699</v>
+        <v>0.0005066018964157468</v>
       </c>
       <c r="E41" t="n">
-        <v>1.005978314702213</v>
+        <v>0.982330849332648</v>
       </c>
       <c r="F41" t="n">
         <v>2</v>
@@ -13127,10 +13127,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>9.590420831201207</v>
+        <v>9.585097992271169</v>
       </c>
       <c r="F4" t="n">
-        <v>0.07125864630213932</v>
+        <v>0.07158376964777426</v>
       </c>
       <c r="G4" t="n">
         <v>2</v>
@@ -13189,10 +13189,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>9.594127399291319</v>
+        <v>9.594526223055531</v>
       </c>
       <c r="F6" t="n">
-        <v>0.07356916788660182</v>
+        <v>0.07343624026828315</v>
       </c>
       <c r="G6" t="n">
         <v>2</v>
@@ -13220,10 +13220,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>9.490588326138381</v>
+        <v>9.578922967016807</v>
       </c>
       <c r="F7" t="n">
-        <v>0.07307501104522025</v>
+        <v>0.07198955589891159</v>
       </c>
       <c r="G7" t="n">
         <v>2</v>
@@ -13437,10 +13437,10 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>8.632758263439488</v>
+        <v>9.546169939979233</v>
       </c>
       <c r="F14" t="n">
-        <v>0.07526691081087925</v>
+        <v>0.07278163777075337</v>
       </c>
       <c r="G14" t="n">
         <v>2</v>
@@ -13654,10 +13654,10 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>9.493832508718906</v>
+        <v>9.584179293364748</v>
       </c>
       <c r="F21" t="n">
-        <v>0.07551523051566378</v>
+        <v>0.07351881448148859</v>
       </c>
       <c r="G21" t="n">
         <v>2</v>
@@ -13871,10 +13871,10 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>8.595416989277203</v>
+        <v>9.579066206968839</v>
       </c>
       <c r="F28" t="n">
-        <v>0.09892150610792125</v>
+        <v>0.08581470533852917</v>
       </c>
       <c r="G28" t="n">
         <v>2</v>
@@ -14088,10 +14088,10 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>9.42610627692604</v>
+        <v>9.55576642150622</v>
       </c>
       <c r="F35" t="n">
-        <v>0.08158106937533811</v>
+        <v>0.07379433397341045</v>
       </c>
       <c r="G35" t="n">
         <v>2</v>
@@ -14305,10 +14305,10 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>7.921074374343686</v>
+        <v>9.111152006374756</v>
       </c>
       <c r="F42" t="n">
-        <v>0.1783748695410168</v>
+        <v>0.09457437701279921</v>
       </c>
       <c r="G42" t="n">
         <v>2</v>
@@ -14356,7 +14356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14415,6 +14415,11 @@
           <t>B_CI_hi</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Mean_N_obs</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -14458,6 +14463,9 @@
       <c r="K2" t="n">
         <v>100</v>
       </c>
+      <c r="L2" t="n">
+        <v>32321</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -14501,6 +14509,9 @@
       <c r="K3" t="n">
         <v>100</v>
       </c>
+      <c r="L3" t="n">
+        <v>29383</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -14544,6 +14555,9 @@
       <c r="K4" t="n">
         <v>100</v>
       </c>
+      <c r="L4" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -14587,6 +14601,9 @@
       <c r="K5" t="n">
         <v>100</v>
       </c>
+      <c r="L5" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -14630,6 +14647,9 @@
       <c r="K6" t="n">
         <v>100</v>
       </c>
+      <c r="L6" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -14673,6 +14693,9 @@
       <c r="K7" t="n">
         <v>100</v>
       </c>
+      <c r="L7" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -14716,6 +14739,9 @@
       <c r="K8" t="n">
         <v>100</v>
       </c>
+      <c r="L8" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -14759,6 +14785,9 @@
       <c r="K9" t="n">
         <v>100</v>
       </c>
+      <c r="L9" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -14802,6 +14831,9 @@
       <c r="K10" t="n">
         <v>100</v>
       </c>
+      <c r="L10" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -14845,6 +14877,9 @@
       <c r="K11" t="n">
         <v>100</v>
       </c>
+      <c r="L11" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -14888,6 +14923,9 @@
       <c r="K12" t="n">
         <v>100</v>
       </c>
+      <c r="L12" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -14931,6 +14969,9 @@
       <c r="K13" t="n">
         <v>100</v>
       </c>
+      <c r="L13" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -14974,6 +15015,9 @@
       <c r="K14" t="n">
         <v>100</v>
       </c>
+      <c r="L14" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -15017,6 +15061,9 @@
       <c r="K15" t="n">
         <v>100</v>
       </c>
+      <c r="L15" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -15060,6 +15107,9 @@
       <c r="K16" t="n">
         <v>100</v>
       </c>
+      <c r="L16" t="n">
+        <v>32321</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -15103,6 +15153,9 @@
       <c r="K17" t="n">
         <v>100</v>
       </c>
+      <c r="L17" t="n">
+        <v>29383</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -15146,6 +15199,9 @@
       <c r="K18" t="n">
         <v>100</v>
       </c>
+      <c r="L18" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -15189,6 +15245,9 @@
       <c r="K19" t="n">
         <v>100</v>
       </c>
+      <c r="L19" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -15232,6 +15291,9 @@
       <c r="K20" t="n">
         <v>100</v>
       </c>
+      <c r="L20" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -15275,6 +15337,9 @@
       <c r="K21" t="n">
         <v>100</v>
       </c>
+      <c r="L21" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -15318,6 +15383,9 @@
       <c r="K22" t="n">
         <v>100</v>
       </c>
+      <c r="L22" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -15361,6 +15429,9 @@
       <c r="K23" t="n">
         <v>100</v>
       </c>
+      <c r="L23" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -15404,6 +15475,9 @@
       <c r="K24" t="n">
         <v>100</v>
       </c>
+      <c r="L24" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -15447,6 +15521,9 @@
       <c r="K25" t="n">
         <v>100</v>
       </c>
+      <c r="L25" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -15490,6 +15567,9 @@
       <c r="K26" t="n">
         <v>100</v>
       </c>
+      <c r="L26" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -15533,6 +15613,9 @@
       <c r="K27" t="n">
         <v>100</v>
       </c>
+      <c r="L27" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -15576,6 +15659,9 @@
       <c r="K28" t="n">
         <v>100</v>
       </c>
+      <c r="L28" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -15619,6 +15705,9 @@
       <c r="K29" t="n">
         <v>100</v>
       </c>
+      <c r="L29" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -15662,6 +15751,9 @@
       <c r="K30" t="n">
         <v>100</v>
       </c>
+      <c r="L30" t="n">
+        <v>32321</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -15705,6 +15797,9 @@
       <c r="K31" t="n">
         <v>100</v>
       </c>
+      <c r="L31" t="n">
+        <v>29383</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -15748,6 +15843,9 @@
       <c r="K32" t="n">
         <v>100</v>
       </c>
+      <c r="L32" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -15791,6 +15889,9 @@
       <c r="K33" t="n">
         <v>65.8</v>
       </c>
+      <c r="L33" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -15834,6 +15935,9 @@
       <c r="K34" t="n">
         <v>100</v>
       </c>
+      <c r="L34" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -15877,6 +15981,9 @@
       <c r="K35" t="n">
         <v>100</v>
       </c>
+      <c r="L35" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -15920,6 +16027,9 @@
       <c r="K36" t="n">
         <v>100</v>
       </c>
+      <c r="L36" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -15963,6 +16073,9 @@
       <c r="K37" t="n">
         <v>100</v>
       </c>
+      <c r="L37" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -16006,6 +16119,9 @@
       <c r="K38" t="n">
         <v>100</v>
       </c>
+      <c r="L38" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -16049,6 +16165,9 @@
       <c r="K39" t="n">
         <v>100</v>
       </c>
+      <c r="L39" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -16092,6 +16211,9 @@
       <c r="K40" t="n">
         <v>100</v>
       </c>
+      <c r="L40" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -16118,22 +16240,25 @@
         <v>2</v>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I41" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>34.2</v>
       </c>
       <c r="K41" t="n">
-        <v>65.8</v>
+        <v>100</v>
+      </c>
+      <c r="L41" t="n">
+        <v>32647</v>
       </c>
     </row>
     <row r="42">
@@ -16178,6 +16303,9 @@
       <c r="K42" t="n">
         <v>100</v>
       </c>
+      <c r="L42" t="n">
+        <v>32647</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -16220,6 +16348,9 @@
       </c>
       <c r="K43" t="n">
         <v>100</v>
+      </c>
+      <c r="L43" t="n">
+        <v>32647</v>
       </c>
     </row>
   </sheetData>

</xml_diff>